<commit_message>
Revert "Wire DSCR/Gross Leverage into live formulas; populate spreading workbook from state"
This reverts commit 0d9d2ae31c379907ff7523829556a8011d28b088.
</commit_message>
<xml_diff>
--- a/templates/spreading/default_spreading_template.xlsx
+++ b/templates/spreading/default_spreading_template.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -615,124 +615,112 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Scheduled Principal Repayment</t>
+          <t>Exceptional Costs / (Income)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Exceptional Costs / (Income)</t>
-        </is>
+          <t>Profit Before Tax</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>B11-B14+B15-B16</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>C11-C14+C15-C16</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>D11-D14+D15-D16</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Profit Before Tax</t>
-        </is>
-      </c>
-      <c r="B18">
-        <f>B11-B14+B15-B17</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>C11-C14+C15-C17</f>
-        <v/>
-      </c>
-      <c r="D18">
-        <f>D11-D14+D15-D17</f>
-        <v/>
+          <t>Tax</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tax</t>
-        </is>
+          <t>Net Profit</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>B17-B18</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>C17-C18</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>D17-D18</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Net Profit</t>
-        </is>
-      </c>
-      <c r="B20">
-        <f>B18-B19</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>C18-C19</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>D18-D19</f>
-        <v/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Key Ratios</t>
+        </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Key Ratios</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DSCR</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DSCR</t>
+          <t>EBIT/Interest</t>
         </is>
       </c>
       <c r="B22">
-        <f>IFERROR(B13/(B14+B16),0)</f>
+        <f>IFERROR(B11/B14,0)</f>
         <v/>
       </c>
       <c r="C22">
-        <f>IFERROR(C13/(C14+C16),0)</f>
+        <f>IFERROR(C11/C14,0)</f>
         <v/>
       </c>
       <c r="D22">
-        <f>IFERROR(D13/(D14+D16),0)</f>
+        <f>IFERROR(D11/D14,0)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EBIT/Interest</t>
+          <t>EBITDA/Interest</t>
         </is>
       </c>
       <c r="B23">
-        <f>IFERROR(B11/B14,0)</f>
+        <f>IFERROR(B13/B14,0)</f>
         <v/>
       </c>
       <c r="C23">
-        <f>IFERROR(C11/C14,0)</f>
+        <f>IFERROR(C13/C14,0)</f>
         <v/>
       </c>
       <c r="D23">
-        <f>IFERROR(D11/D14,0)</f>
+        <f>IFERROR(D13/D14,0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EBITDA/Interest</t>
-        </is>
-      </c>
-      <c r="B24">
-        <f>IFERROR(B13/B14,0)</f>
-        <v/>
-      </c>
-      <c r="C24">
-        <f>IFERROR(C13/C14,0)</f>
-        <v/>
-      </c>
-      <c r="D24">
-        <f>IFERROR(D13/D14,0)</f>
-        <v/>
+          <t>Gross Leverage</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -770,15 +758,15 @@
         </is>
       </c>
       <c r="B29">
-        <f>B26+B27+B28</f>
+        <f>SUM(B26:B28)</f>
         <v/>
       </c>
       <c r="C29">
-        <f>C26+C27+C28</f>
+        <f>SUM(C26:C28)</f>
         <v/>
       </c>
       <c r="D29">
-        <f>D26+D27+D28</f>
+        <f>SUM(D26:D28)</f>
         <v/>
       </c>
     </row>
@@ -817,15 +805,15 @@
         </is>
       </c>
       <c r="B34">
-        <f>B30+B31+B32+B33</f>
+        <f>SUM(B30:B33)</f>
         <v/>
       </c>
       <c r="C34">
-        <f>C30+C31+C32+C33</f>
+        <f>SUM(C30:C33)</f>
         <v/>
       </c>
       <c r="D34">
-        <f>D30+D31+D32+D33</f>
+        <f>SUM(D30:D33)</f>
         <v/>
       </c>
     </row>
@@ -883,15 +871,15 @@
         </is>
       </c>
       <c r="B40">
-        <f>B36+B37+B38+B39</f>
+        <f>SUM(B36:B39)</f>
         <v/>
       </c>
       <c r="C40">
-        <f>C36+C37+C38+C39</f>
+        <f>SUM(C36:C39)</f>
         <v/>
       </c>
       <c r="D40">
-        <f>D36+D37+D38+D39</f>
+        <f>SUM(D36:D39)</f>
         <v/>
       </c>
     </row>
@@ -930,15 +918,15 @@
         </is>
       </c>
       <c r="B45">
-        <f>B41+B42+B43+B44</f>
+        <f>SUM(B41:B44)</f>
         <v/>
       </c>
       <c r="C45">
-        <f>C41+C42+C43+C44</f>
+        <f>SUM(C41:C44)</f>
         <v/>
       </c>
       <c r="D45">
-        <f>D41+D42+D43+D44</f>
+        <f>SUM(D41:D44)</f>
         <v/>
       </c>
     </row>
@@ -982,15 +970,15 @@
         </is>
       </c>
       <c r="B49">
-        <f>B47+B48</f>
+        <f>SUM(B47:B48)</f>
         <v/>
       </c>
       <c r="C49">
-        <f>C47+C48</f>
+        <f>SUM(C47:C48)</f>
         <v/>
       </c>
       <c r="D49">
-        <f>D47+D48</f>
+        <f>SUM(D47:D48)</f>
         <v/>
       </c>
     </row>
@@ -1078,68 +1066,49 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Gross Leverage</t>
-        </is>
-      </c>
-      <c r="B55">
-        <f>IFERROR((B37+B38+B41+B42)/B13,0)</f>
-        <v/>
-      </c>
-      <c r="C55">
-        <f>IFERROR((C37+C38+C41+C42)/C13,0)</f>
-        <v/>
-      </c>
-      <c r="D55">
-        <f>IFERROR((D37+D38+D41+D42)/D13,0)</f>
-        <v/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Working Capital</t>
+        </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Working Capital</t>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Trade Debtor Days</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Trade Debtor Days</t>
+          <t>Trade Creditor Days</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Trade Creditor Days</t>
+          <t>Stock Days</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Stock Days</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
           <t>Working Capital Cycle (days)</t>
         </is>
       </c>
-      <c r="B60">
-        <f>B57+B59-B58</f>
-        <v/>
-      </c>
-      <c r="C60">
-        <f>C57+C59-C58</f>
-        <v/>
-      </c>
-      <c r="D60">
-        <f>D57+D59-D58</f>
+      <c r="B59">
+        <f>B56+B58-B57</f>
+        <v/>
+      </c>
+      <c r="C59">
+        <f>C56+C58-C57</f>
+        <v/>
+      </c>
+      <c r="D59">
+        <f>D56+D58-D57</f>
         <v/>
       </c>
     </row>
@@ -1154,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1165,7 +1134,6 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1209,13 +1177,13 @@
           <t>CV % of Exposure</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Perfection Status</t>
-        </is>
-      </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[Asset class]</t>
+        </is>
+      </c>
       <c r="H2">
         <f>IFERROR(G2/B2,0)</f>
         <v/>

</xml_diff>